<commit_message>
ADD: Projeto do controle de loudness
Simulação, relatório e link de compra do potenciometro
</commit_message>
<xml_diff>
--- a/Compras/Compras.xlsx
+++ b/Compras/Compras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rafael\UFRJ\TCC\Compras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFCF8455-91FA-4615-AE26-0E0A115C9AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF84C086-5912-4174-AB7F-D1BA0C94EB9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{18DE3399-BDB8-455B-A1D0-3EF492C640E0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Link</t>
   </si>
@@ -65,7 +65,16 @@
     <t>Observação</t>
   </si>
   <si>
-    <t>AmpOp</t>
+    <t>Potenciômetro com tap</t>
+  </si>
+  <si>
+    <t>https://pt.aliexpress.com/item/1005006031222394.html?spm=a2g0o.tesla.0.0.1705kaArkaArFi&amp;pdp_npi=5%40dis%21BRL%21R%2411%2C02%21R%249%2C36%21%21%21%21%21%402101c5b217557224093411492e6cfa%2112000043414867971%21btf%21%21%21%211%210&amp;afTraceInfo=1005006031222394__pc__c_ppc_item_bridge_pc_main__tD3IKeD__1755722409431&amp;gatewayAdapt=glo2bra</t>
+  </si>
+  <si>
+    <t>Ali Express</t>
+  </si>
+  <si>
+    <t>Pré-Amp</t>
   </si>
 </sst>
 </file>
@@ -75,7 +84,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,6 +96,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -295,48 +312,49 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -348,8 +366,12 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -728,16 +750,28 @@
       <c r="B6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
+      <c r="C6" s="11">
+        <v>1</v>
+      </c>
+      <c r="D6" s="12">
+        <v>9.36</v>
+      </c>
+      <c r="E6" s="12">
+        <v>23.71</v>
+      </c>
       <c r="F6" s="12">
         <f>C6*D6+E6</f>
-        <v>0</v>
-      </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
+        <v>33.07</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="J6" s="13"/>
     </row>
     <row r="7" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -1035,6 +1069,9 @@
       <c r="J27" s="9"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H6" r:id="rId1" display="https://pt.aliexpress.com/item/1005006031222394.html?spm=a2g0o.tesla.0.0.1705kaArkaArFi&amp;pdp_npi=5%40dis%21BRL%21R%2411%2C02%21R%249%2C36%21%21%21%21%21%402101c5b217557224093411492e6cfa%2112000043414867971%21btf%21%21%21%211%210&amp;afTraceInfo=1005006031222394__pc__c_ppc_item_bridge_pc_main__tD3IKeD__1755722409431&amp;gatewayAdapt=glo2bra" xr:uid="{47324D1E-D6C4-43AF-BE0D-9FCCCB921809}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>